<commit_message>
Update config.json and Daily Economic Report
</commit_message>
<xml_diff>
--- a/Stock_Analyzer/Daily_Economic_Report_20260622.xlsx
+++ b/Stock_Analyzer/Daily_Economic_Report_20260622.xlsx
@@ -2401,17 +2401,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wed, 17 Jun 2026 20:23:30 GMT</t>
+          <t>Sun, 21 Jun 2026 09:45:05 GMT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>v.daum.net</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>美, '워시체제' 첫 FOMC서 금리 또 동결…연내 인하→인상 전환(종합2보)</t>
+          <t>[주간 증시전망] 코스피시장 대형주 접근이 바람직</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2421,24 +2421,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1XNE1JVVJkeWNqXzFSSWZkUEhVbmtOZnhCR1M4ZmpvdTcwbEZjZk5DSzg4aUhfM3JwMS0xUXh5WWR4YU1HUWpxdVNubGxWdWZ0SlVROFVhVFhERmvSAWBBVV95cUxQWkpRdy1WWUE2clA0U2VHNjVhbEtIQl9EUUFKUmxBNThncWRXRTk2Y0UydzV3RDhrenYtX1NRdDNlaUtaUW5LMXBsMkJSbDhrT2FWZk1BUThhLVFZdjI2YU4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE96UDdKTENSWTJSYS1EVlFncDNIN0lHelVuY29EMzdwenlfN3RxalBhaDhtYVZ1Ni15bG1CUkJTaUY0RE1XdVFzUlUtVDQyT0U?oc=5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wed, 17 Jun 2026 18:49:00 GMT</t>
+          <t>Sun, 21 Jun 2026 08:35:55 GMT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>한국경제</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>연준, 금리 동결했지만 전망 엇갈려...트럼프 "괜찮다"</t>
+          <t>뉴욕·상하이 증시, 美·이란 후속 협상에 뉴욕증시 '촉각'</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2448,14 +2448,14 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE5mX3VoSDNqTU1hek01WHl0YVBLMVFpaF80YmdoNkh0X2t0VjJlNFNrdkRvOVpuVmdsSGhXOGNOZzVfdW9XdllTN1JWajlUanZRRnZXT21FMUY5WGZMc3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE0tTlZUQVNZRElraEZuaHJSZ2o0S3pZTHJlbl9ZU1JZelEtTVdzOG5yeEg4aW1oVEJnWEpWNEtoWDk2TDU5ZlVEeU9zU1AxaEstWDFFb2MxVFFHUdIBVEFVX3lxTE5lYmI5dVVGSjY1S0pacWhxZ3hTMTdiQWpyTDA2RHczS2VsQUdFc2tqOUpZWUo5RDJHbUwxNVVaQWhpaFR6eFpub2s5MGlBRnNyaDI1WA?oc=5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sun, 21 Jun 2026 09:45:05 GMT</t>
+          <t>Sun, 21 Jun 2026 15:08:36 GMT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[주간 증시전망] 코스피시장 대형주 접근이 바람직</t>
+          <t>[월요마당] 통계는 나침반, 경제총조사가 방향을 잡는다</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2475,14 +2475,14 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE96UDdKTENSWTJSYS1EVlFncDNIN0lHelVuY29EMzdwenlfN3RxalBhaDhtYVZ1Ni15bG1CUkJTaUY0RE1XdVFzUlUtVDQyT0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE05ZVpMSWtqeTczMGJuY3I2Si14TllZZFhvLVpJeld3Q3RzSnpoRjlEM09JY0VPMUswRGUzY3VQTUlSYTRidV8xQUotem5aZmc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sun, 21 Jun 2026 08:35:55 GMT</t>
+          <t>Sun, 21 Jun 2026 08:58:44 GMT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>뉴욕·상하이 증시, 美·이란 후속 협상에 뉴욕증시 '촉각'</t>
+          <t>재테크의 모든 것 '한경 머니로드쇼'</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE0tTlZUQVNZRElraEZuaHJSZ2o0S3pZTHJlbl9ZU1JZelEtTVdzOG5yeEg4aW1oVEJnWEpWNEtoWDk2TDU5ZlVEeU9zU1AxaEstWDFFb2MxVFFHUdIBVEFVX3lxTE5lYmI5dVVGSjY1S0pacWhxZ3hTMTdiQWpyTDA2RHczS2VsQUdFc2tqOUpZWUo5RDJHbUwxNVVaQWhpaFR6eFpub2s5MGlBRnNyaDI1WA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9vQnlnUW1hb2NOcEc1RWNiaVgwU1pZaXFoVktnRGZJZXZVWXdpU0IxNS1GMG01eUlmdWZDeUJodUNsYV9OSkdNQng0a0tfeW9ISHlfSmRWSExUQdIBVEFVX3lxTFBPSDhHRGE2eFZOMkFnNWdjWlZpdjQ2RXY0aHpDT0Fkam1qUHI3a0lKR0MwM2lKOGlaeDNnZ3kxRW1FcjVsejhTby1yeFJrMlBOZmsxdA?oc=5</t>
         </is>
       </c>
     </row>
@@ -2536,17 +2536,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sun, 21 Jun 2026 08:58:44 GMT</t>
+          <t>Sun, 21 Jun 2026 07:08:16 GMT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>v.daum.net</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>재테크의 모든 것 '한경 머니로드쇼'</t>
+          <t>코스피 9000인데 국내 증시 8%가 동전주…7월부터 상장폐지 대상 올라</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2556,14 +2556,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9vQnlnUW1hb2NOcEc1RWNiaVgwU1pZaXFoVktnRGZJZXZVWXdpU0IxNS1GMG01eUlmdWZDeUJodUNsYV9OSkdNQng0a0tfeW9ISHlfSmRWSExUQdIBVEFVX3lxTFBPSDhHRGE2eFZOMkFnNWdjWlZpdjQ2RXY0aHpDT0Fkam1qUHI3a0lKR0MwM2lKOGlaeDNnZ3kxRW1FcjVsejhTby1yeFJrMlBOZmsxdA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE11RUdNN280aU9rOGxKSGRaeXdmbkhjTDRfUFM1azVFOUFORkVPUjFCNHFzcldaMjFwbmFGaGMwNmJrR25NYm1KUTZUYUdiV2c?oc=5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sun, 21 Jun 2026 07:08:16 GMT</t>
+          <t>Sun, 21 Jun 2026 01:17:19 GMT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>코스피 9000인데 국내 증시 8%가 동전주…7월부터 상장폐지 대상 올라</t>
+          <t>미국 연내 금리인상 가능성 ‘↑’…9000 찍은 코스피엔 불리하다 ‘경고’</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2583,14 +2583,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE11RUdNN280aU9rOGxKSGRaeXdmbkhjTDRfUFM1azVFOUFORkVPUjFCNHFzcldaMjFwbmFGaGMwNmJrR25NYm1KUTZUYUdiV2c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiRkFVX3lxTE94a2E2d3FfRm94WDd2d2NpTDFYLXpjSHF4V3pSRzg0bVgxd1d0dXA0ejdDb1J6WkxpQ3hZWEhENGE4Z2E3Qnc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sun, 21 Jun 2026 01:17:19 GMT</t>
+          <t>Sun, 21 Jun 2026 15:21:18 GMT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>미국 연내 금리인상 가능성 ‘↑’…9000 찍은 코스피엔 불리하다 ‘경고’</t>
+          <t>‘MSCI 선진국’ 노리는 韓증시… 23일 관찰대상국 발표</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiRkFVX3lxTE94a2E2d3FfRm94WDd2d2NpTDFYLXpjSHF4V3pSRzg0bVgxd1d0dXA0ejdDb1J6WkxpQ3hZWEhENGE4Z2E3Qnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiT0FVX3lxTE4yUEdIR3JaSWt2djQzSC15UVR4S1hEd1V6TlYydFl5cGdNdzhXOEd2OTQ3YnVDSjhHMW1BUmtja0ZWWTdDenZMaWU2UVBTSmM?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>